<commit_message>
Updates to block diagram showing PoE and new BOM components in the right place.
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>Component</t>
   </si>
@@ -84,24 +84,6 @@
     <t>IP67-rated waterproof housing with mounting plate</t>
   </si>
   <si>
-    <t>Internal RF Pigtail</t>
-  </si>
-  <si>
-    <t>RG-316 IPEX to N-Female</t>
-  </si>
-  <si>
-    <t>Bulkhead connector to bridge booster to enclosure wall</t>
-  </si>
-  <si>
-    <t>Exterior Low-Loss Coax</t>
-  </si>
-  <si>
-    <t>LMR-400 (3ft)</t>
-  </si>
-  <si>
-    <t>Double-shielded ultra low-loss cable for 1W signal</t>
-  </si>
-  <si>
     <t>High-Gain Antenna</t>
   </si>
   <si>
@@ -166,6 +148,33 @@
   </si>
   <si>
     <t>30dBm Power Amplifier with Integrated LNA requiring 5VDC supply</t>
+  </si>
+  <si>
+    <t>UFLMMCX10</t>
+  </si>
+  <si>
+    <t>100MMCXSMAFBH3</t>
+  </si>
+  <si>
+    <t>UFLSMA6</t>
+  </si>
+  <si>
+    <t>RAK4631 → 915MPA Cable</t>
+  </si>
+  <si>
+    <t>u.FL/IPEX (MHF1) plug → MMCX male, R/A, 10"</t>
+  </si>
+  <si>
+    <t>915MPA antenna → SMA cable</t>
+  </si>
+  <si>
+    <t>RAK4631 → antenna amp bypass</t>
+  </si>
+  <si>
+    <t>u.FL/IPEX (MHF1) plug → SMA female bulkhead w/ O-ring, 6"</t>
+  </si>
+  <si>
+    <t>MMCX male, R/A → SMA female bulkhead w/ O-ring, RG316, 3"</t>
   </si>
 </sst>
 </file>
@@ -985,10 +994,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="76.7109375" bestFit="1" customWidth="1"/>
   </cols>
@@ -1043,7 +1052,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D4" s="1">
         <v>1</v>
@@ -1092,28 +1101,28 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8">
+      <c r="A8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="D9" s="1">
         <v>1</v>
@@ -1121,13 +1130,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="C10" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D10" s="1">
         <v>1</v>
@@ -1135,13 +1144,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="D11" s="1">
         <v>1</v>
@@ -1149,41 +1158,41 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D12" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C13" t="s">
-        <v>35</v>
-      </c>
-      <c r="D13">
+      <c r="A13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B14" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="C14" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -1191,13 +1200,13 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C15" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -1205,15 +1214,29 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="B16" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="C16" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="D16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17">
         <v>1</v>
       </c>
     </row>

</xml_diff>